<commit_message>
Trotter mesh: supplier schedule keeps received, ending inventory and cut PO columns
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WMbR8uWBiFLctZQqB3wnd7
</commit_message>
<xml_diff>
--- a/Mesh cutting supplier (Trotter)/Trotter_6-Month_Schedule.xlsx
+++ b/Mesh cutting supplier (Trotter)/Trotter_6-Month_Schedule.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="ddd mm/dd/yy"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="ddd mm/dd/yy"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -59,7 +60,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +70,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1B2A41"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -118,41 +124,44 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -520,15 +529,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="64" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -558,490 +570,657 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>Received (pcs)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Ending inventory (pcs)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Cut PO released (rolls)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
           <t>Trotter actions</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Rolls at Trotter (start of week)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Roll order (rolls shipped by Intuitive)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="13" t="n">
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="4" t="n">
         <v>46293</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>837</v>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="6" t="n">
+        <v>587</v>
+      </c>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Our 3 rolls in transit to you (5 bd)</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="G5" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>Intuitive releases PO-0 (1 roll, 1,300 pcs) and ships 3 rolls on 9/24</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="13" t="n">
+      <c r="A6" s="4" t="n">
         <v>46300</v>
       </c>
       <c r="B6" s="5" t="n">
         <v>587</v>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="6" t="n">
+        <v>337</v>
+      </c>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Receive 3 rolls (5 bd)</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="G6" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="6" t="inlineStr"/>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="8" t="inlineStr"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="13" t="n">
+      <c r="A7" s="4" t="n">
         <v>46307</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>337</v>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="6" t="n">
+        <v>87</v>
+      </c>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>Cut PO-0 (1,300 pcs) and ship (2 bd)</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="G7" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="6" t="inlineStr"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="8" t="inlineStr"/>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="4" t="n">
         <v>46314</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="5" t="n">
         <v>87</v>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="11" t="n">
+        <v>-163</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>PO-0 in transit to Intuitive (5 bd); Cut PO-1 (1,300 pcs) and ship (2 bd)</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="G8" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="11" t="inlineStr">
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="13" t="inlineStr">
         <is>
           <t>Intuitive stock runs out ~Tue 10/20; PO-0 arrives ~Tue 10/20 — please ship PO-0 as early as you can. Intuitive releases PO-1 (1 roll)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="13" t="n">
+      <c r="A9" s="4" t="n">
         <v>46321</v>
       </c>
-      <c r="B9" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="B9" s="5" t="n">
+        <v>-163</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>1300</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>887</v>
+      </c>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>PO-1 in transit to Intuitive (5 bd)</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="G9" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="11" t="inlineStr">
-        <is>
-          <t>PO-0 received at Intuitive. Intuitive short ~163 pcs until PO-0 arrives</t>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>PO-0 received at Intuitive</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="13" t="n">
+      <c r="A10" s="4" t="n">
         <v>46328</v>
       </c>
       <c r="B10" s="5" t="n">
         <v>887</v>
       </c>
-      <c r="C10" s="6" t="inlineStr"/>
-      <c r="D10" s="7" t="n">
+      <c r="C10" s="14" t="n">
+        <v>1300</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>1937</v>
+      </c>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="8" t="inlineStr"/>
+      <c r="G10" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>PO-1 received at Intuitive</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="13" t="n">
+      <c r="A11" s="4" t="n">
         <v>46335</v>
       </c>
       <c r="B11" s="5" t="n">
         <v>1937</v>
       </c>
-      <c r="C11" s="6" t="inlineStr"/>
-      <c r="D11" s="7" t="n">
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n">
+        <v>1687</v>
+      </c>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="8" t="inlineStr"/>
+      <c r="G11" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="6" t="inlineStr"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="8" t="inlineStr"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="13" t="n">
+      <c r="A12" s="4" t="n">
         <v>46342</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>1687</v>
       </c>
-      <c r="C12" s="6" t="inlineStr"/>
-      <c r="D12" s="7" t="n">
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n">
+        <v>1437</v>
+      </c>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="8" t="inlineStr"/>
+      <c r="G12" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="6" t="inlineStr"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="8" t="inlineStr"/>
     </row>
     <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="13" t="n">
+      <c r="A13" s="4" t="n">
         <v>46349</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>1437</v>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n">
+        <v>1187</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>Cut PO-2 (1,300 pcs) and ship (2 bd)</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="G13" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>Intuitive releases PO-2 (1 roll). Thanksgiving week — please confirm you are open</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="13" t="n">
+      <c r="A14" s="4" t="n">
         <v>46356</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>1187</v>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n">
+        <v>937</v>
+      </c>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>PO-2 in transit to Intuitive (5 bd)</t>
         </is>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="G14" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="6" t="inlineStr"/>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="8" t="inlineStr"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="13" t="n">
+      <c r="A15" s="4" t="n">
         <v>46363</v>
       </c>
       <c r="B15" s="5" t="n">
         <v>937</v>
       </c>
-      <c r="C15" s="6" t="inlineStr"/>
-      <c r="D15" s="7" t="n">
+      <c r="C15" s="14" t="n">
+        <v>1300</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>1987</v>
+      </c>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="8" t="inlineStr"/>
+      <c r="G15" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="8" t="inlineStr">
         <is>
           <t>PO-2 received at Intuitive</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="13" t="n">
+      <c r="A16" s="4" t="n">
         <v>46370</v>
       </c>
       <c r="B16" s="5" t="n">
         <v>1987</v>
       </c>
-      <c r="C16" s="6" t="inlineStr"/>
-      <c r="D16" s="7" t="n">
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n">
+        <v>1737</v>
+      </c>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="8" t="inlineStr"/>
+      <c r="G16" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="6" t="inlineStr"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="8" t="inlineStr"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="13" t="n">
+      <c r="A17" s="4" t="n">
         <v>46377</v>
       </c>
       <c r="B17" s="5" t="n">
         <v>1737</v>
       </c>
-      <c r="C17" s="6" t="inlineStr"/>
-      <c r="D17" s="7" t="n">
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n">
+        <v>1487</v>
+      </c>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="8" t="inlineStr"/>
+      <c r="G17" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="H17" s="7" t="n"/>
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>Christmas week — please confirm closures</t>
         </is>
       </c>
     </row>
     <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="13" t="n">
+      <c r="A18" s="4" t="n">
         <v>46384</v>
       </c>
       <c r="B18" s="5" t="n">
         <v>1487</v>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n">
+        <v>1237</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>Cut PO-3 (1,300 pcs) and ship (2 bd); Our 3 rolls in transit to you (5 bd)</t>
         </is>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="G18" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="H18" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Intuitive releases PO-3 (1 roll). Intuitive orders and ships 3 rolls (fills your 3-roll storage). New Year week — please confirm closures</t>
         </is>
       </c>
     </row>
     <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="13" t="n">
+      <c r="A19" s="4" t="n">
         <v>46391</v>
       </c>
       <c r="B19" s="5" t="n">
         <v>1237</v>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n">
+        <v>987</v>
+      </c>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>PO-3 in transit to Intuitive (5 bd); Receive 3 rolls (5 bd)</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="G19" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="7" t="n"/>
-      <c r="F19" s="6" t="inlineStr"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="8" t="inlineStr"/>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="13" t="n">
+      <c r="A20" s="4" t="n">
         <v>46398</v>
       </c>
       <c r="B20" s="5" t="n">
         <v>987</v>
       </c>
-      <c r="C20" s="6" t="inlineStr"/>
-      <c r="D20" s="7" t="n">
+      <c r="C20" s="14" t="n">
+        <v>1300</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>2037</v>
+      </c>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="8" t="inlineStr"/>
+      <c r="G20" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="H20" s="7" t="n"/>
+      <c r="I20" s="8" t="inlineStr">
         <is>
           <t>PO-3 received at Intuitive</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="13" t="n">
+      <c r="A21" s="4" t="n">
         <v>46405</v>
       </c>
       <c r="B21" s="5" t="n">
         <v>2037</v>
       </c>
-      <c r="C21" s="6" t="inlineStr"/>
-      <c r="D21" s="7" t="n">
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n">
+        <v>1787</v>
+      </c>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="8" t="inlineStr"/>
+      <c r="G21" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E21" s="7" t="n"/>
-      <c r="F21" s="6" t="inlineStr"/>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="8" t="inlineStr"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="13" t="n">
+      <c r="A22" s="4" t="n">
         <v>46412</v>
       </c>
       <c r="B22" s="5" t="n">
         <v>1787</v>
       </c>
-      <c r="C22" s="6" t="inlineStr"/>
-      <c r="D22" s="7" t="n">
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n">
+        <v>1537</v>
+      </c>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="8" t="inlineStr"/>
+      <c r="G22" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="6" t="inlineStr"/>
+      <c r="H22" s="7" t="n"/>
+      <c r="I22" s="8" t="inlineStr"/>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="13" t="n">
+      <c r="A23" s="4" t="n">
         <v>46419</v>
       </c>
       <c r="B23" s="5" t="n">
         <v>1537</v>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n">
+        <v>1287</v>
+      </c>
+      <c r="E23" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
         <is>
           <t>Cut PO-4 (1,300 pcs) and ship (2 bd)</t>
         </is>
       </c>
-      <c r="D23" s="7" t="n">
+      <c r="G23" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>Intuitive releases PO-4 (1 roll)</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="13" t="n">
+      <c r="A24" s="4" t="n">
         <v>46426</v>
       </c>
       <c r="B24" s="5" t="n">
         <v>1287</v>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="n">
+        <v>1037</v>
+      </c>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>PO-4 in transit to Intuitive (5 bd)</t>
         </is>
       </c>
-      <c r="D24" s="7" t="n">
+      <c r="G24" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E24" s="7" t="n"/>
-      <c r="F24" s="6" t="inlineStr"/>
+      <c r="H24" s="7" t="n"/>
+      <c r="I24" s="8" t="inlineStr"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="13" t="n">
+      <c r="A25" s="4" t="n">
         <v>46433</v>
       </c>
       <c r="B25" s="5" t="n">
         <v>1037</v>
       </c>
-      <c r="C25" s="6" t="inlineStr"/>
-      <c r="D25" s="7" t="n">
+      <c r="C25" s="14" t="n">
+        <v>1300</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>2087</v>
+      </c>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="8" t="inlineStr"/>
+      <c r="G25" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E25" s="7" t="n"/>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="H25" s="7" t="n"/>
+      <c r="I25" s="8" t="inlineStr">
         <is>
           <t>PO-4 received at Intuitive</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="13" t="n">
+      <c r="A26" s="4" t="n">
         <v>46440</v>
       </c>
       <c r="B26" s="5" t="n">
         <v>2087</v>
       </c>
-      <c r="C26" s="6" t="inlineStr"/>
-      <c r="D26" s="7" t="n">
+      <c r="C26" s="5" t="n"/>
+      <c r="D26" s="5" t="n">
+        <v>1837</v>
+      </c>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="8" t="inlineStr"/>
+      <c r="G26" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E26" s="7" t="n"/>
-      <c r="F26" s="6" t="inlineStr"/>
+      <c r="H26" s="7" t="n"/>
+      <c r="I26" s="8" t="inlineStr"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="13" t="n">
+      <c r="A27" s="4" t="n">
         <v>46447</v>
       </c>
       <c r="B27" s="5" t="n">
         <v>1837</v>
       </c>
-      <c r="C27" s="6" t="inlineStr"/>
-      <c r="D27" s="7" t="n">
+      <c r="C27" s="5" t="n"/>
+      <c r="D27" s="5" t="n">
+        <v>1587</v>
+      </c>
+      <c r="E27" s="7" t="n"/>
+      <c r="F27" s="8" t="inlineStr"/>
+      <c r="G27" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E27" s="7" t="n"/>
-      <c r="F27" s="6" t="inlineStr"/>
+      <c r="H27" s="7" t="n"/>
+      <c r="I27" s="8" t="inlineStr"/>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="13" t="n">
+      <c r="A28" s="4" t="n">
         <v>46454</v>
       </c>
       <c r="B28" s="5" t="n">
         <v>1587</v>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C28" s="5" t="n"/>
+      <c r="D28" s="5" t="n">
+        <v>1337</v>
+      </c>
+      <c r="E28" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
         <is>
           <t>Cut PO-5 (1,300 pcs) and ship (2 bd)</t>
         </is>
       </c>
-      <c r="D28" s="7" t="n">
+      <c r="G28" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E28" s="7" t="n"/>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="H28" s="7" t="n"/>
+      <c r="I28" s="8" t="inlineStr">
         <is>
           <t>Intuitive releases PO-5 (1 roll)</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="13" t="n">
+      <c r="A29" s="4" t="n">
         <v>46461</v>
       </c>
       <c r="B29" s="5" t="n">
         <v>1337</v>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="n">
+        <v>1087</v>
+      </c>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="8" t="inlineStr">
         <is>
           <t>PO-5 in transit to Intuitive (5 bd)</t>
         </is>
       </c>
-      <c r="D29" s="7" t="n">
+      <c r="G29" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E29" s="7" t="n"/>
-      <c r="F29" s="6" t="inlineStr"/>
+      <c r="H29" s="7" t="n"/>
+      <c r="I29" s="8" t="inlineStr"/>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="13" t="n">
+      <c r="A30" s="4" t="n">
         <v>46468</v>
       </c>
       <c r="B30" s="5" t="n">
         <v>1087</v>
       </c>
-      <c r="C30" s="6" t="inlineStr"/>
-      <c r="D30" s="7" t="n">
+      <c r="C30" s="14" t="n">
+        <v>1300</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>2137</v>
+      </c>
+      <c r="E30" s="7" t="n"/>
+      <c r="F30" s="8" t="inlineStr"/>
+      <c r="G30" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="7" t="n"/>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="H30" s="7" t="n"/>
+      <c r="I30" s="8" t="inlineStr">
         <is>
           <t>PO-5 received at Intuitive</t>
         </is>
@@ -1050,12 +1229,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Green = Trotter cuts and ships that week · Blue = Trotter receives rolls · Yellow = Intuitive ships rolls to Trotter · Red = Intuitive stock at risk. Inventory figures are Intuitive Surgical planning estimates.</t>
+          <t>Yellow = PO / roll order released · Green = Trotter cuts and ships · Blue = receipt · Red = Intuitive stock below zero, pale yellow = below the 2-box minimum (867 pcs). Inventory figures are Intuitive Surgical planning estimates.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>